<commit_message>
feat: add general photo evaluation category
</commit_message>
<xml_diff>
--- a/app/public/fixtures/checklist-import-template.xlsx
+++ b/app/public/fixtures/checklist-import-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>路线顺序</t>
   </si>
@@ -40,6 +40,9 @@
     <t>好的表述</t>
   </si>
   <si>
+    <t>一般表现表述</t>
+  </si>
+  <si>
     <t>提醒表述</t>
   </si>
   <si>
@@ -74,6 +77,9 @@
   </si>
   <si>
     <t>检查标准第1项（原编号1）落实较好。</t>
+  </si>
+  <si>
+    <t>检查标准第1项（原编号1）7S管理基本落实，但现场标准仍有提升空间。</t>
   </si>
   <si>
     <t>检查标准第1项（原编号1）落实不到位，本次予以提醒。</t>
@@ -466,13 +472,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="13" width="20" customWidth="1"/>
+    <col min="1" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,46 +518,52 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="N2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>